<commit_message>
Increase learning rate in OPGD update for enhanced convergence speed
</commit_message>
<xml_diff>
--- a/multi_regression/figs_100/regression_result.xlsx
+++ b/multi_regression/figs_100/regression_result.xlsx
@@ -598,22 +598,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0.6953 $\pm$ 0.3471</t>
+          <t>0.3280 $\pm$ 0.1003</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2.2459 $\pm$ 0.5407</t>
+          <t>0.9663 $\pm$ 0.1773</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0.7338 $\pm$ 0.3784</t>
+          <t>0.4428 $\pm$ 0.0860</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>0.7254 $\pm$ 0.3588</t>
+          <t>0.3926 $\pm$ 0.0871</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update learning rate in synthetic strategic prediction for improved performance
</commit_message>
<xml_diff>
--- a/multi_regression/figs_100/regression_result.xlsx
+++ b/multi_regression/figs_100/regression_result.xlsx
@@ -571,22 +571,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>4.4387 $\pm$ 2.4365</t>
+          <t>3.9956 $\pm$ 2.1163</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.1360 $\pm$ 3.0144</t>
+          <t>4.3717 $\pm$ 3.4092</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>3.3390 $\pm$ 1.5476</t>
+          <t>3.6357 $\pm$ 2.0388</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>4.0282 $\pm$ 2.1750</t>
+          <t>3.8324 $\pm$ 2.1366</t>
         </is>
       </c>
     </row>

</xml_diff>